<commit_message>
Update various PDF and SQL files with new content and improved clarity
</commit_message>
<xml_diff>
--- a/batch_notes/batch_27.xlsx
+++ b/batch_notes/batch_27.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10625"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10630"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/ALI_2/work/acciojob/modules/sql/postgresql/batch_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D5FFD1-C178-564C-84CD-919CB93B6A02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3B9F901-EB91-C14A-9818-06E0620802EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29400" yWindow="-2480" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{43D057EC-24A4-D14F-BD50-FDFE67984E9E}"/>
+    <workbookView xWindow="29400" yWindow="-2480" windowWidth="38400" windowHeight="21600" activeTab="3" xr2:uid="{43D057EC-24A4-D14F-BD50-FDFE67984E9E}"/>
   </bookViews>
   <sheets>
     <sheet name="01" sheetId="1" r:id="rId1"/>
     <sheet name="03" sheetId="2" r:id="rId2"/>
+    <sheet name="04" sheetId="3" r:id="rId3"/>
+    <sheet name="05" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="129">
   <si>
     <t>RDBMS</t>
   </si>
@@ -172,6 +174,261 @@
   </si>
   <si>
     <t>INTERVAL</t>
+  </si>
+  <si>
+    <t>user_id</t>
+  </si>
+  <si>
+    <t>manually</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>error</t>
+  </si>
+  <si>
+    <t>Error</t>
+  </si>
+  <si>
+    <t>serial | PK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">serial </t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Bicycle</t>
+  </si>
+  <si>
+    <t>Pen</t>
+  </si>
+  <si>
+    <t>NULL</t>
+  </si>
+  <si>
+    <t>Unique</t>
+  </si>
+  <si>
+    <t>Primary Key</t>
+  </si>
+  <si>
+    <t>Unique + Not Null + Reference</t>
+  </si>
+  <si>
+    <t>Foreign Key</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>emp_id</t>
+  </si>
+  <si>
+    <t>emp_name</t>
+  </si>
+  <si>
+    <t>emp_address</t>
+  </si>
+  <si>
+    <t>Salary</t>
+  </si>
+  <si>
+    <t>salary_id</t>
+  </si>
+  <si>
+    <t>salary</t>
+  </si>
+  <si>
+    <t>PK</t>
+  </si>
+  <si>
+    <t>FK</t>
+  </si>
+  <si>
+    <t>Salary_history</t>
+  </si>
+  <si>
+    <t>orderf_items</t>
+  </si>
+  <si>
+    <t>order_id</t>
+  </si>
+  <si>
+    <t>prod_id</t>
+  </si>
+  <si>
+    <t>Emp_id</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>E0001</t>
+  </si>
+  <si>
+    <t>Cat</t>
+  </si>
+  <si>
+    <t>cat_id</t>
+  </si>
+  <si>
+    <t>cat_name</t>
+  </si>
+  <si>
+    <t>brand</t>
+  </si>
+  <si>
+    <t>brand_id</t>
+  </si>
+  <si>
+    <t>brand_name</t>
+  </si>
+  <si>
+    <t>Parent</t>
+  </si>
+  <si>
+    <t>Child</t>
+  </si>
+  <si>
+    <t>cat</t>
+  </si>
+  <si>
+    <t>Orphan</t>
+  </si>
+  <si>
+    <t>DELETE 3</t>
+  </si>
+  <si>
+    <t>CASCADE</t>
+  </si>
+  <si>
+    <t>Force something which was restricted</t>
+  </si>
+  <si>
+    <t>DELETE from table</t>
+  </si>
+  <si>
+    <t>delete from table cascade</t>
+  </si>
+  <si>
+    <t>violating foreign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Default </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ON delete </t>
+  </si>
+  <si>
+    <t>Restricted</t>
+  </si>
+  <si>
+    <t>Don’t allow delete</t>
+  </si>
+  <si>
+    <t>Cascade</t>
+  </si>
+  <si>
+    <t>It will delete all child records</t>
+  </si>
+  <si>
+    <t>on delete</t>
+  </si>
+  <si>
+    <t>Set NULL</t>
+  </si>
+  <si>
+    <t>When pareent is deleted set all child to null</t>
+  </si>
+  <si>
+    <t>It will forcefullly delete parent but will not touch child at all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop </t>
+  </si>
+  <si>
+    <t>Order Placed</t>
+  </si>
+  <si>
+    <t>Lucknow</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>Seller</t>
+  </si>
+  <si>
+    <t>Kanyakumari</t>
+  </si>
+  <si>
+    <t>Land</t>
+  </si>
+  <si>
+    <t>Storage</t>
+  </si>
+  <si>
+    <t>Blueprint</t>
+  </si>
+  <si>
+    <t>Fill Products</t>
+  </si>
+  <si>
+    <t>Remove Products</t>
+  </si>
+  <si>
+    <t>Update Products</t>
+  </si>
+  <si>
+    <t>DML</t>
+  </si>
+  <si>
+    <t>insert</t>
+  </si>
+  <si>
+    <t>delete</t>
+  </si>
+  <si>
+    <t>update</t>
+  </si>
+  <si>
+    <t>Retrieval of product</t>
+  </si>
+  <si>
+    <t>DQL</t>
+  </si>
+  <si>
+    <t>select</t>
+  </si>
+  <si>
+    <t>DCL</t>
+  </si>
+  <si>
+    <t>Grant</t>
+  </si>
+  <si>
+    <t>Revoke</t>
+  </si>
+  <si>
+    <t>TCL</t>
+  </si>
+  <si>
+    <t>Begin</t>
+  </si>
+  <si>
+    <t>Commit</t>
+  </si>
+  <si>
+    <t>rollback</t>
+  </si>
+  <si>
+    <t>Savepoint</t>
   </si>
 </sst>
 </file>
@@ -187,15 +444,39 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -240,17 +521,117 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1527,6 +1908,103 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>428020</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>146840</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>202140</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>114520</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="2" name="Ink 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0EB9ABD-D895-BA56-C8C9-ADE3F8F34863}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="1253520" y="8884440"/>
+            <a:ext cx="5006520" cy="780480"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="2" name="Ink 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0EB9ABD-D895-BA56-C8C9-ADE3F8F34863}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="1249200" y="8880120"/>
+              <a:ext cx="5015160" cy="789120"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/ink/ink1.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-07-02T16:09:00.977"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.025" units="cm"/>
+      <inkml:brushProperty name="height" value="0.025" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1 379 24575,'4'2'0,"0"18"0,4 3 0,2 32 0,1 18 0,-6-8 0,-1 5 0,-1-4 0,-2 1 0,-2 12 0,-2-2 0,-2-21 0,0-4 0,-1 31 0,-3-39 0,9-14 0,0-22 0,0 0 0,0 0 0,2-4 0,0 1 0,27 2 0,53 18 0,0-7 0,-15-4 0,16 0 0,-15-5 0,10 1 0,8-1 0,4 0 0,4 0-869,-5-2 0,5-2 0,4 1 0,4-1 0,1 0 1,1 1-1,0 0 869,-15 0 0,2 1 0,1 0 0,1 0 0,1 0 0,0 0 0,1 0 0,-1-1 0,1 0 0,4-1 0,1 0 0,2 0 0,1-1 0,-1 0 0,-2 0 0,-2-1 0,-3 1 0,-4-1 0,15 0 0,-3 1 0,-4-1 0,-3-1 0,-5 0 0,-3 1 0,9-1 0,-5 0 0,-6-1 0,-6 0 0,-5-1 0,-5 0 0,-14 0 0,5 5 0,-11 4 0,5 3 0,27 11 0,5 2 0,-10-6 0,7 1 0,-12-2 0,9 3 0,0-1 0,-8-4-335,11 0 1,0-4 334,-15-2 0,7 0 0,3 0 0,-3-3 0,15-2 0,-1-2 0,5-1 0,-18 0 0,4 0 0,2 1 0,1-1 0,0-1 395,0 0 0,0-1 0,1 0 1,0 1-1,2 0-395,6 2 0,2 1 0,1 0 0,-2 1 0,-1 0 0,-7 0 0,0 0 0,-2 0 0,-2 1 0,-4 0-351,3 1 0,-4 0 1,-1 1-1,0 2 351,4 4 0,1 3 0,-1 0 0,-7-2 0,-3-4 0,-5-1 0,5 2 0,5 6 0,5 2 0,4 1 0,4-5 0,-4-6 0,5-4 0,2-1 0,0-1 0,-1 2 0,-1 1 0,-1 2 0,1 0 0,-1-1 0,0-1 0,-1-3 0,1 0 0,-1-2 0,-2-1 0,-5-2 0,26-2 0,-6-4 0,-12-2 0,-14-3 0,-7-2 0,1 1 0,-5-2 697,24-26-697,-30 17 0,-4 6 0,7 0 0,19 1 0,11 1 431,-13 4 1,9 2-1,5-1 1,-2 1-432,1-1 0,0 1 0,2 0 0,6-2 0,-14 2 0,6-1 0,3-1 0,0 0 0,-3 0 0,-4-1 0,15-2 0,-4-2 0,-4 1 0,-4 1 504,11-1 0,-5 1 0,-12-1-504,-6-4 0,-25 6 0,-45 14 0,-3-2 0,0 2 0,2 0 2100,-2-6-2100,5-1 143,5-8-143,35-41 0,-6-7 0,8-18 0,-1-8 0,-18 17 0,-4 0 0,11-13 0,-5 3 0,-19 27 0,-5 8 0,0-2 0,-16 23 0,-4 11 0,-8 3 0,-6-6 0,-3 1 0,6 3 0,-2-1 0,8 2 0,-1-2 0,1 2 0,9 3 0,0 6 0,0-2 0,-2 5 0,-6-4 0,3 3 0,-1-1 0,4 1 0,-2 4 0,1 0 0,3 2 0,1 4 0,-6 21 0,-8 20 0,6 0 0,-4-8 0,17-25 0,-10 4 0,6-11 0,-4 9 0,21-48 0,24-30 0,12-14 0,-12 17 0,1-4 0,4-2 0,1 2 0,5-4 0,-1 0 0,-3 5 0,0-1 0,-2 4 0,-2 4 0,15-12 0,-9 13 0,-14 16 0,-14 24 0,-13 11 0,-3 8 0,2 2 0,1 8 0,1 34 0,5 32 0,-4-34 0,0 4 0,0 21 0,0 3 0,-2-3 0,-1 0 0,-5 7 0,-2 0 0,3-6 0,-2-7 0,-6 7 0,8-29 0,0-40 0,0 0 0,0 0 0,0-2 0,0 0 0</inkml:trace>
+</inkml:ink>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B75C81F2-16C4-AA43-AAFC-971767DED54C}" name="Table1" displayName="Table1" ref="C6:C13" totalsRowShown="0">
   <autoFilter ref="C6:C13" xr:uid="{B75C81F2-16C4-AA43-AAFC-971767DED54C}"/>
@@ -2073,7 +2551,7 @@
     <row r="20" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C20" s="5">
         <f ca="1">NOW()</f>
-        <v>46201.50655046296</v>
+        <v>46205.957528356485</v>
       </c>
     </row>
     <row r="21" spans="3:7" x14ac:dyDescent="0.2">
@@ -2107,4 +2585,959 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2C6501E-B810-AE4F-88C4-7F4CA8CAF68B}">
+  <dimension ref="B2:L105"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C11">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C13" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="H24" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="H25" t="s">
+        <v>52</v>
+      </c>
+      <c r="J25" s="7"/>
+    </row>
+    <row r="26" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="H26" t="s">
+        <v>53</v>
+      </c>
+      <c r="J26" s="7"/>
+      <c r="L26" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="H27" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="H28" t="s">
+        <v>55</v>
+      </c>
+      <c r="J28" s="8"/>
+    </row>
+    <row r="29" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="H29" t="s">
+        <v>55</v>
+      </c>
+      <c r="J29" s="8"/>
+      <c r="L29" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+    </row>
+    <row r="32" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="H36" t="s">
+        <v>58</v>
+      </c>
+      <c r="J36" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="J37" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B38" s="6"/>
+      <c r="C38" s="6"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="6"/>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="6"/>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>60</v>
+      </c>
+      <c r="G42" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="44" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
+        <v>61</v>
+      </c>
+      <c r="C44" t="s">
+        <v>62</v>
+      </c>
+      <c r="D44" t="s">
+        <v>63</v>
+      </c>
+      <c r="G44" t="s">
+        <v>65</v>
+      </c>
+      <c r="H44" t="s">
+        <v>61</v>
+      </c>
+      <c r="I44" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
+        <v>67</v>
+      </c>
+      <c r="G45" t="s">
+        <v>67</v>
+      </c>
+      <c r="H45" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="48" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="H48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G52" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G54" t="s">
+        <v>65</v>
+      </c>
+      <c r="H54" t="s">
+        <v>61</v>
+      </c>
+      <c r="I54" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G55" t="s">
+        <v>67</v>
+      </c>
+      <c r="H55" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="H56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="H57">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B58" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B59" t="s">
+        <v>71</v>
+      </c>
+      <c r="C59" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B60" t="s">
+        <v>55</v>
+      </c>
+      <c r="C60">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B61" t="s">
+        <v>55</v>
+      </c>
+      <c r="C61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B64" t="s">
+        <v>73</v>
+      </c>
+      <c r="F64" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="65" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B65" t="s">
+        <v>67</v>
+      </c>
+      <c r="F65" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="66" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B66" t="s">
+        <v>16</v>
+      </c>
+      <c r="C66">
+        <v>1</v>
+      </c>
+      <c r="F66" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="67" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B67" t="s">
+        <v>74</v>
+      </c>
+      <c r="C67" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="70" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B70" t="s">
+        <v>76</v>
+      </c>
+      <c r="E70" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="71" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B71" t="s">
+        <v>77</v>
+      </c>
+      <c r="C71" t="s">
+        <v>78</v>
+      </c>
+      <c r="E71" t="s">
+        <v>80</v>
+      </c>
+      <c r="F71" t="s">
+        <v>81</v>
+      </c>
+      <c r="G71" t="s">
+        <v>77</v>
+      </c>
+      <c r="I71" t="s">
+        <v>82</v>
+      </c>
+      <c r="J71" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="72" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B72" t="s">
+        <v>67</v>
+      </c>
+      <c r="E72" t="s">
+        <v>67</v>
+      </c>
+      <c r="G72" t="s">
+        <v>68</v>
+      </c>
+      <c r="I72" t="s">
+        <v>84</v>
+      </c>
+      <c r="J72" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="73" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="E73">
+        <v>1</v>
+      </c>
+      <c r="G73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B74">
+        <v>2</v>
+      </c>
+      <c r="E74">
+        <v>2</v>
+      </c>
+      <c r="G74">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B75">
+        <v>3</v>
+      </c>
+      <c r="E75">
+        <v>3</v>
+      </c>
+      <c r="G75">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="76" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="E76">
+        <v>4</v>
+      </c>
+      <c r="G76">
+        <v>3</v>
+      </c>
+      <c r="I76" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="81" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B81" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="84" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B84" t="s">
+        <v>87</v>
+      </c>
+      <c r="C84" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="88" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G88" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="89" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B89" t="s">
+        <v>89</v>
+      </c>
+      <c r="D89" t="s">
+        <v>91</v>
+      </c>
+      <c r="E89" t="s">
+        <v>92</v>
+      </c>
+      <c r="F89" t="s">
+        <v>93</v>
+      </c>
+      <c r="H89" t="s">
+        <v>94</v>
+      </c>
+      <c r="I89" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="90" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G90" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="92" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G92" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="93" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="F93" t="s">
+        <v>93</v>
+      </c>
+      <c r="H93" t="s">
+        <v>96</v>
+      </c>
+      <c r="I93" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="94" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G94" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="96" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G96" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="97" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="F97" t="s">
+        <v>98</v>
+      </c>
+      <c r="H97" t="s">
+        <v>99</v>
+      </c>
+      <c r="I97" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="98" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="G98" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="102" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B102" t="s">
+        <v>90</v>
+      </c>
+      <c r="I102" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="J102" s="9"/>
+      <c r="K102" s="9"/>
+    </row>
+    <row r="103" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B103" t="s">
+        <v>102</v>
+      </c>
+      <c r="I103" s="9"/>
+      <c r="J103" s="9"/>
+      <c r="K103" s="9"/>
+    </row>
+    <row r="104" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="I104" s="9"/>
+      <c r="J104" s="9"/>
+      <c r="K104" s="9"/>
+    </row>
+    <row r="105" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="I105" s="9"/>
+      <c r="J105" s="9"/>
+      <c r="K105" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I102:K105"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{588172D2-80C2-1542-89AB-245B6BCA7E13}">
+  <dimension ref="B2:O23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="4.33203125" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="C4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="D5" t="s">
+        <v>105</v>
+      </c>
+      <c r="E5" t="s">
+        <v>106</v>
+      </c>
+      <c r="F5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D7" s="12"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="14"/>
+      <c r="N7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="D8" s="15"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="17"/>
+    </row>
+    <row r="9" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D9" s="15"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="17"/>
+      <c r="N9" t="s">
+        <v>110</v>
+      </c>
+      <c r="O9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="D10" s="15"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="17"/>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>111</v>
+      </c>
+      <c r="D11" s="15"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
+      <c r="I11" s="16"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="16"/>
+      <c r="L11" s="17"/>
+      <c r="N11" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="O11" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>112</v>
+      </c>
+      <c r="D12" s="15"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="17"/>
+      <c r="N12" s="9"/>
+      <c r="O12" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>113</v>
+      </c>
+      <c r="D13" s="15"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="17"/>
+      <c r="N13" s="9"/>
+      <c r="O13" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="D14" s="15"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="17"/>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="D15" s="15"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="17"/>
+      <c r="N15" t="s">
+        <v>119</v>
+      </c>
+      <c r="O15" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>118</v>
+      </c>
+      <c r="D16" s="15"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="17"/>
+    </row>
+    <row r="17" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="D17" s="15"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="17"/>
+      <c r="N17" t="s">
+        <v>121</v>
+      </c>
+      <c r="O17" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="D18" s="18"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="19"/>
+      <c r="L18" s="22"/>
+      <c r="O18" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="19" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="D19" s="18"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="22"/>
+    </row>
+    <row r="20" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="D20" s="18"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="22"/>
+      <c r="N20" t="s">
+        <v>124</v>
+      </c>
+      <c r="O20" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="21" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="D21" s="18"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="19"/>
+      <c r="J21" s="19"/>
+      <c r="K21" s="19"/>
+      <c r="L21" s="22"/>
+      <c r="O21" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="22" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="D22" s="18"/>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="19"/>
+      <c r="K22" s="19"/>
+      <c r="L22" s="22"/>
+      <c r="O22" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" spans="4:15" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="D23" s="20"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="21"/>
+      <c r="L23" s="23"/>
+      <c r="O23" t="s">
+        <v>128</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="N11:N13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>